<commit_message>
updated employee turn over with dashboard image
</commit_message>
<xml_diff>
--- a/Employee Turnover Analysis Excel Dashboard Dataset.xlsx
+++ b/Employee Turnover Analysis Excel Dashboard Dataset.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\notes\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70CFE260-4FFF-4B59-957A-A4A858AC5E9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E5ACB52-B659-426E-AEF8-DD04F3690A3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,9 +16,10 @@
     <sheet name="Sheet3" sheetId="3" r:id="rId1"/>
     <sheet name="Sheet1" sheetId="1" r:id="rId2"/>
     <sheet name="Sheet5" sheetId="7" r:id="rId3"/>
-    <sheet name="dashboard1" sheetId="2" r:id="rId4"/>
-    <sheet name="dashboard2" sheetId="5" r:id="rId5"/>
-    <sheet name="exit reasons" sheetId="6" r:id="rId6"/>
+    <sheet name="Sheet6" sheetId="8" r:id="rId4"/>
+    <sheet name="dashboard1" sheetId="2" r:id="rId5"/>
+    <sheet name="dashboard2" sheetId="5" r:id="rId6"/>
+    <sheet name="exit reasons" sheetId="6" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="age_wise_record_pivot">dashboard1!$D$13:$F$19</definedName>
@@ -28,9 +29,9 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="2" r:id="rId7"/>
-    <pivotCache cacheId="1" r:id="rId8"/>
-    <pivotCache cacheId="7" r:id="rId9"/>
+    <pivotCache cacheId="2" r:id="rId8"/>
+    <pivotCache cacheId="1" r:id="rId9"/>
+    <pivotCache cacheId="7" r:id="rId10"/>
   </pivotCaches>
 </workbook>
 </file>
@@ -12520,6 +12521,15 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C651C4B1-600F-409C-93FA-696A6126E827}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4FBFEBF7-E327-4F24-AFA8-CCB4AB4E943C}">
   <dimension ref="A1:J29"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -12992,7 +13002,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A3CD709-3FE1-49EF-A208-1E8C06F38C03}">
   <dimension ref="C14:C16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -13009,7 +13019,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CFFEBE0D-0B57-4060-AE3D-65B48591CFF3}">
   <dimension ref="A1:L2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>